<commit_message>
Alinhar banco ao exame CAM: mercadorias e passageiros, filtros por tema
</commit_message>
<xml_diff>
--- a/questoes sem rep.xlsx
+++ b/questoes sem rep.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J212"/>
+  <dimension ref="A1:K212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,11 @@
           <t>notas_revisao</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>tema_exame</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -509,6 +514,11 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -546,7 +556,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Capacidade financeira (IMT/DL 257/2007): 9.000 € no 1.º veículo; 5.000 € (pesado) ou 900 € (ligeiro) por cada veículo adicional.</t>
+          <t>Resposta aceite no exame (DL 257/2007 / IMT): 9.000 € no 1.º veículo; 5.000 € (pesado) ou 900 € (ligeiro) por veículo adicional.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -557,6 +567,11 @@
       <c r="J3" t="inlineStr">
         <is>
           <t>Corrigido valor do veículo ligeiro: 1.500 € → 900 € (fonte: imt-ip.pt).</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
         </is>
       </c>
     </row>
@@ -601,6 +616,11 @@
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -643,6 +663,11 @@
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -685,6 +710,11 @@
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -727,6 +757,11 @@
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -769,6 +804,11 @@
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -811,6 +851,11 @@
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -853,6 +898,11 @@
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -895,6 +945,11 @@
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -937,6 +992,11 @@
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -979,6 +1039,11 @@
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1021,6 +1086,11 @@
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1063,6 +1133,11 @@
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1105,6 +1180,11 @@
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1147,6 +1227,11 @@
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1189,6 +1274,11 @@
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1231,6 +1321,11 @@
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1273,6 +1368,11 @@
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1315,6 +1415,11 @@
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1357,6 +1462,11 @@
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1399,6 +1509,11 @@
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1441,6 +1556,11 @@
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1483,6 +1603,11 @@
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1525,6 +1650,11 @@
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1567,6 +1697,11 @@
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1609,6 +1744,11 @@
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1651,6 +1791,11 @@
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1693,6 +1838,11 @@
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1735,6 +1885,11 @@
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1777,6 +1932,11 @@
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1819,6 +1979,11 @@
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1861,6 +2026,11 @@
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1903,6 +2073,11 @@
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1945,6 +2120,11 @@
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1987,6 +2167,11 @@
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2029,6 +2214,11 @@
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2071,6 +2261,11 @@
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2113,6 +2308,11 @@
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2155,6 +2355,11 @@
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2197,6 +2402,11 @@
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2239,6 +2449,11 @@
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2281,6 +2496,11 @@
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2323,6 +2543,11 @@
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2365,6 +2590,11 @@
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2407,6 +2637,11 @@
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2449,6 +2684,11 @@
       </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2491,6 +2731,11 @@
       </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2533,6 +2778,11 @@
       </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2575,6 +2825,11 @@
       </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2617,6 +2872,11 @@
       </c>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2659,6 +2919,11 @@
       </c>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2701,6 +2966,11 @@
       </c>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2743,6 +3013,11 @@
       </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2785,6 +3060,11 @@
       </c>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2827,6 +3107,11 @@
       </c>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2869,6 +3154,11 @@
       </c>
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2911,6 +3201,11 @@
       </c>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2953,6 +3248,11 @@
       </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2995,6 +3295,11 @@
       </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3037,6 +3342,11 @@
       </c>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3079,6 +3389,11 @@
       </c>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3121,6 +3436,11 @@
       </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3163,6 +3483,11 @@
       </c>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3205,6 +3530,11 @@
       </c>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3247,6 +3577,11 @@
       </c>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3289,6 +3624,11 @@
       </c>
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3331,6 +3671,11 @@
       </c>
       <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3373,6 +3718,11 @@
       </c>
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>passageiros</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3415,6 +3765,11 @@
       </c>
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3457,6 +3812,11 @@
       </c>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3499,6 +3859,11 @@
       </c>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3541,6 +3906,11 @@
       </c>
       <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3583,6 +3953,11 @@
       </c>
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3625,6 +4000,11 @@
       </c>
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3667,6 +4047,11 @@
       </c>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3709,6 +4094,11 @@
       </c>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3751,6 +4141,11 @@
       </c>
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3793,6 +4188,11 @@
       </c>
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3835,6 +4235,11 @@
       </c>
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3877,6 +4282,11 @@
       </c>
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3919,6 +4329,11 @@
       </c>
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3961,6 +4376,11 @@
       </c>
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -4003,6 +4423,11 @@
       </c>
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -4045,6 +4470,11 @@
       </c>
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -4087,6 +4517,11 @@
       </c>
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4129,6 +4564,11 @@
       </c>
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4171,6 +4611,11 @@
       </c>
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4211,14 +4656,11 @@
           <t>É crime e pode acarretar sanções pesadas.</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -4263,6 +4705,11 @@
       </c>
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4305,6 +4752,11 @@
       </c>
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4347,6 +4799,11 @@
       </c>
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4389,6 +4846,11 @@
       </c>
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4431,6 +4893,11 @@
       </c>
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4473,6 +4940,11 @@
       </c>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4515,6 +4987,11 @@
       </c>
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4557,6 +5034,11 @@
       </c>
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -4599,6 +5081,11 @@
       </c>
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -4641,6 +5128,11 @@
       </c>
       <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4683,6 +5175,11 @@
       </c>
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -4723,14 +5220,11 @@
           <t>É crime com sanções pesadas.</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -4775,6 +5269,11 @@
       </c>
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -4817,6 +5316,11 @@
       </c>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -4859,6 +5363,11 @@
       </c>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -4901,6 +5410,11 @@
       </c>
       <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -4943,6 +5457,11 @@
       </c>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -4985,6 +5504,11 @@
       </c>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -5027,6 +5551,11 @@
       </c>
       <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -5069,6 +5598,11 @@
       </c>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -5111,6 +5645,11 @@
       </c>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -5153,6 +5692,11 @@
       </c>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -5195,6 +5739,11 @@
       </c>
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -5237,6 +5786,11 @@
       </c>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -5279,6 +5833,11 @@
       </c>
       <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -5321,6 +5880,11 @@
       </c>
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -5363,6 +5927,11 @@
       </c>
       <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -5405,6 +5974,11 @@
       </c>
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -5447,6 +6021,11 @@
       </c>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -5489,6 +6068,11 @@
       </c>
       <c r="I120" t="inlineStr"/>
       <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -5531,6 +6115,11 @@
       </c>
       <c r="I121" t="inlineStr"/>
       <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -5573,6 +6162,11 @@
       </c>
       <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -5615,6 +6209,11 @@
       </c>
       <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -5657,6 +6256,11 @@
       </c>
       <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -5699,6 +6303,11 @@
       </c>
       <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -5741,6 +6350,11 @@
       </c>
       <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -5781,14 +6395,11 @@
           <t>Podem ser bilhetes simples ou passes/assina tura.</t>
         </is>
       </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -5831,14 +6442,11 @@
           <t>Uniforme e apresentação cuidada são obrigatórios.</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -5883,6 +6491,11 @@
       </c>
       <c r="I129" t="inlineStr"/>
       <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>passageiros</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -5923,14 +6536,11 @@
           <t>Até 20 kg de bagagem por passageiro é gratuito.</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J130" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -5975,6 +6585,11 @@
       </c>
       <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -6017,6 +6632,11 @@
       </c>
       <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -6057,14 +6677,11 @@
           <t>Transportes públicos bons = menos carros na estrada = menos poluição.</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J133" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -6107,14 +6724,11 @@
           <t>Em Portugal, o transporte rodoviário é o mais usado.</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J134" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -6157,14 +6771,11 @@
           <t>Pode ser por conta própria ou por conta de outrem.</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J135" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>
@@ -6209,6 +6820,11 @@
       </c>
       <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -6249,14 +6865,11 @@
           <t>Tem de ser alguém com responsabilidade efetiva na gestão.</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>
@@ -6299,14 +6912,11 @@
           <t>Várias formas jurídicas são permitidas.</t>
         </is>
       </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -6349,14 +6959,11 @@
           <t>Alvará ou licença comunitária válida até 5 anos.</t>
         </is>
       </c>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J139" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>
@@ -6399,14 +7006,11 @@
           <t>Contrato escrito com a entidade que contrata o serviço.</t>
         </is>
       </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J140" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -6451,6 +7055,11 @@
       </c>
       <c r="I141" t="inlineStr"/>
       <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -6493,6 +7102,11 @@
       </c>
       <c r="I142" t="inlineStr"/>
       <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -6535,6 +7149,11 @@
       </c>
       <c r="I143" t="inlineStr"/>
       <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -6577,6 +7196,11 @@
       </c>
       <c r="I144" t="inlineStr"/>
       <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -6617,14 +7241,11 @@
           <t>Serviços regulares = horários e tarifas fixos.</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J145" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -6669,6 +7290,11 @@
       </c>
       <c r="I146" t="inlineStr"/>
       <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -6711,12 +7337,17 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>corrigida; revisar_escopo</t>
+          <t>corrigida</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>Preenchida opção D em falta. Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+          <t>Preenchida opção D em falta.</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>
@@ -6761,6 +7392,11 @@
       </c>
       <c r="I148" t="inlineStr"/>
       <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -6803,6 +7439,11 @@
       </c>
       <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -6845,6 +7486,11 @@
       </c>
       <c r="I150" t="inlineStr"/>
       <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -6887,6 +7533,11 @@
       </c>
       <c r="I151" t="inlineStr"/>
       <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -6929,6 +7580,11 @@
       </c>
       <c r="I152" t="inlineStr"/>
       <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -6971,6 +7627,11 @@
       </c>
       <c r="I153" t="inlineStr"/>
       <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -7013,6 +7674,11 @@
       </c>
       <c r="I154" t="inlineStr"/>
       <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -7055,6 +7721,11 @@
       </c>
       <c r="I155" t="inlineStr"/>
       <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -7097,6 +7768,11 @@
       </c>
       <c r="I156" t="inlineStr"/>
       <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -7139,6 +7815,11 @@
       </c>
       <c r="I157" t="inlineStr"/>
       <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -7181,6 +7862,11 @@
       </c>
       <c r="I158" t="inlineStr"/>
       <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -7223,6 +7909,11 @@
       </c>
       <c r="I159" t="inlineStr"/>
       <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>misto</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -7265,6 +7956,11 @@
       </c>
       <c r="I160" t="inlineStr"/>
       <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -7307,6 +8003,11 @@
       </c>
       <c r="I161" t="inlineStr"/>
       <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -7349,6 +8050,11 @@
       </c>
       <c r="I162" t="inlineStr"/>
       <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -7399,6 +8105,11 @@
           <t>Preenchida opção D em falta.</t>
         </is>
       </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -7436,7 +8147,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>O airbag é complementar ao cinto de segurança; usado isoladamente pode causar lesões. Todas as afirmações são verdadeiras.</t>
+          <t>Resposta aceite no exame: todas as afirmações sobre o airbag são verdadeiras.</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -7447,6 +8158,11 @@
       <c r="J164" t="inlineStr">
         <is>
           <t>Resposta corrigida D→C; opção D preenchida.</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>comum</t>
         </is>
       </c>
     </row>
@@ -7499,6 +8215,11 @@
           <t>Preenchida opção C em falta.</t>
         </is>
       </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -7541,6 +8262,11 @@
       </c>
       <c r="I166" t="inlineStr"/>
       <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -7583,6 +8309,11 @@
       </c>
       <c r="I167" t="inlineStr"/>
       <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -7625,6 +8356,11 @@
       </c>
       <c r="I168" t="inlineStr"/>
       <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -7667,6 +8403,11 @@
       </c>
       <c r="I169" t="inlineStr"/>
       <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -7709,6 +8450,11 @@
       </c>
       <c r="I170" t="inlineStr"/>
       <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -7759,6 +8505,11 @@
           <t>Preenchida opção D em falta.</t>
         </is>
       </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -7801,6 +8552,11 @@
       </c>
       <c r="I172" t="inlineStr"/>
       <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -7843,6 +8599,11 @@
       </c>
       <c r="I173" t="inlineStr"/>
       <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -7885,6 +8646,11 @@
       </c>
       <c r="I174" t="inlineStr"/>
       <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -7927,6 +8693,11 @@
       </c>
       <c r="I175" t="inlineStr"/>
       <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -7977,6 +8748,11 @@
           <t>Preenchida opção D em falta.</t>
         </is>
       </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -8019,6 +8795,11 @@
       </c>
       <c r="I177" t="inlineStr"/>
       <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -8061,6 +8842,11 @@
       </c>
       <c r="I178" t="inlineStr"/>
       <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>mercadorias</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -8103,6 +8889,11 @@
       </c>
       <c r="I179" t="inlineStr"/>
       <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -8145,6 +8936,11 @@
       </c>
       <c r="I180" t="inlineStr"/>
       <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>passageiros</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -8187,6 +8983,11 @@
       </c>
       <c r="I181" t="inlineStr"/>
       <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -8229,6 +9030,11 @@
       </c>
       <c r="I182" t="inlineStr"/>
       <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -8271,6 +9077,11 @@
       </c>
       <c r="I183" t="inlineStr"/>
       <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -8313,6 +9124,11 @@
       </c>
       <c r="I184" t="inlineStr"/>
       <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -8355,6 +9171,11 @@
       </c>
       <c r="I185" t="inlineStr"/>
       <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -8397,6 +9218,11 @@
       </c>
       <c r="I186" t="inlineStr"/>
       <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -8439,6 +9265,11 @@
       </c>
       <c r="I187" t="inlineStr"/>
       <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -8479,14 +9310,11 @@
           <t>Autocarro articulado 4+ eixos = 32 toneladas.</t>
         </is>
       </c>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J188" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -8529,14 +9357,11 @@
           <t>Veículo &gt; 4 anos = inspeção anual.</t>
         </is>
       </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J189" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -8579,14 +9404,11 @@
           <t>Requisitos de acesso: idoneidade + capacidade profissional + financeira.</t>
         </is>
       </c>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J190" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I190" t="inlineStr"/>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>
@@ -8629,14 +9451,11 @@
           <t>Alta qualidade = 100+ km, categoria III, poucas paragens.</t>
         </is>
       </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J191" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -8679,14 +9498,11 @@
           <t>Falta não suprida em 1 ano = caducidade do alvará.</t>
         </is>
       </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J192" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I192" t="inlineStr"/>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>
@@ -8731,6 +9547,11 @@
       </c>
       <c r="I193" t="inlineStr"/>
       <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -8773,6 +9594,11 @@
       </c>
       <c r="I194" t="inlineStr"/>
       <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -8813,14 +9639,11 @@
           <t>Balanço ou garantia bancária.</t>
         </is>
       </c>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J195" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I195" t="inlineStr"/>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -8863,14 +9686,11 @@
           <t>Não aprovação = caducidade da licença do veículo.</t>
         </is>
       </c>
-      <c r="I196" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J196" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I196" t="inlineStr"/>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -8913,14 +9733,11 @@
           <t>Várias formas jurídicas permitidas.</t>
         </is>
       </c>
-      <c r="I197" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J197" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I197" t="inlineStr"/>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -8960,17 +9777,14 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>Mínimo € 50 000 para início.</t>
-        </is>
-      </c>
-      <c r="I198" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J198" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+          <t>Resposta habitualmente aceite nos testes de passageiros do exame CAM/CP. Confirme sempre com o manual da sua entidade formadora.</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr"/>
+      <c r="J198" t="inlineStr"/>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -9015,6 +9829,11 @@
       </c>
       <c r="I199" t="inlineStr"/>
       <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>passageiros</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -9055,14 +9874,11 @@
           <t>Verificar sempre (acesso e exercício).</t>
         </is>
       </c>
-      <c r="I200" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J200" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I200" t="inlineStr"/>
+      <c r="J200" t="inlineStr"/>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>
@@ -9105,14 +9921,11 @@
           <t>Várias formas de aquisição permitidas.</t>
         </is>
       </c>
-      <c r="I201" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J201" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I201" t="inlineStr"/>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -9157,6 +9970,11 @@
       </c>
       <c r="I202" t="inlineStr"/>
       <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>passageiros</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -9199,6 +10017,11 @@
       </c>
       <c r="I203" t="inlineStr"/>
       <c r="J203" t="inlineStr"/>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>comum</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -9239,14 +10062,11 @@
           <t>Dístico + folha de itinerário.</t>
         </is>
       </c>
-      <c r="I204" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J204" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I204" t="inlineStr"/>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -9289,14 +10109,11 @@
           <t>No pedido de acesso.</t>
         </is>
       </c>
-      <c r="I205" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J205" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I205" t="inlineStr"/>
+      <c r="J205" t="inlineStr"/>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -9339,14 +10156,11 @@
           <t>30 dias, sob pena de coima.</t>
         </is>
       </c>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J206" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I206" t="inlineStr"/>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -9389,14 +10203,11 @@
           <t>Interdição profissional = perda de idoneidade.</t>
         </is>
       </c>
-      <c r="I207" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J207" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I207" t="inlineStr"/>
+      <c r="J207" t="inlineStr"/>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>
@@ -9439,14 +10250,11 @@
           <t>Serviços regulares especializados = categorias específicas.</t>
         </is>
       </c>
-      <c r="I208" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J208" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I208" t="inlineStr"/>
+      <c r="J208" t="inlineStr"/>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -9489,14 +10297,11 @@
           <t>Ocasionais + regulares especializados nacionais.</t>
         </is>
       </c>
-      <c r="I209" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J209" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I209" t="inlineStr"/>
+      <c r="J209" t="inlineStr"/>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>
@@ -9539,14 +10344,11 @@
           <t>Municipais e intermunicipais.</t>
         </is>
       </c>
-      <c r="I210" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J210" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I210" t="inlineStr"/>
+      <c r="J210" t="inlineStr"/>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -9589,14 +10391,11 @@
           <t>Até 20 kg gratuito.</t>
         </is>
       </c>
-      <c r="I211" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J211" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I211" t="inlineStr"/>
+      <c r="J211" t="inlineStr"/>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>passageiros</t>
         </is>
       </c>
     </row>
@@ -9639,14 +10438,11 @@
           <t>Certificado para transportes particulares.</t>
         </is>
       </c>
-      <c r="I212" t="inlineStr">
-        <is>
-          <t>revisar_escopo</t>
-        </is>
-      </c>
-      <c r="J212" t="inlineStr">
-        <is>
-          <t>Questão de transporte de passageiros — verificar relevância para exame CAM mercadorias.</t>
+      <c r="I212" t="inlineStr"/>
+      <c r="J212" t="inlineStr"/>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>misto</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrigir questão 40: amarração em laço resposta B (IMT)
</commit_message>
<xml_diff>
--- a/questoes sem rep.xlsx
+++ b/questoes sem rep.xlsx
@@ -2298,16 +2298,24 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>b</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>A amarração em laço vai de um lado da carroçaria ao outro por cima da carga.</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+          <t>Resposta aceite no exame (IMT): amarração em laço liga a carga a um dos lados da carroçaria, para evitar o deslizamento e a inclinação para o lado oposto. A opção D descreve a amarração de topo.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>corrigida</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Resposta corrigida D-&gt;B (manual IMT Acondicionamento de Carga).</t>
+        </is>
+      </c>
       <c r="K40" t="inlineStr">
         <is>
           <t>mercadorias</t>

</xml_diff>

<commit_message>
Corrigir gabarito questao 75 para A
</commit_message>
<xml_diff>
--- a/questoes sem rep.xlsx
+++ b/questoes sem rep.xlsx
@@ -4169,7 +4169,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>a</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -4177,8 +4177,16 @@
           <t>Aumentar a altura da carga — é o que melhor responde ao enunciado (opção B)).</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>corrigida</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Gabarito corrigido manualmente: A</t>
+        </is>
+      </c>
       <c r="K72" t="inlineStr">
         <is>
           <t>mercadorias</t>

</xml_diff>

<commit_message>
Corrigir gabarito questao 553 para B
</commit_message>
<xml_diff>
--- a/questoes sem rep.xlsx
+++ b/questoes sem rep.xlsx
@@ -24985,7 +24985,7 @@
       </c>
       <c r="G436" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>b</t>
         </is>
       </c>
       <c r="H436" t="inlineStr">
@@ -24995,12 +24995,12 @@
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t>gabarito_testescam</t>
+          <t>corrigida</t>
         </is>
       </c>
       <c r="J436" t="inlineStr">
         <is>
-          <t>Importado IMT rel_2 | Gabarito IMT pendente | Gabarito TestesCAM (exato 100%, opcao_texto)</t>
+          <t>Gabarito corrigido manualmente: B</t>
         </is>
       </c>
       <c r="K436" t="inlineStr">

</xml_diff>

<commit_message>
Corrigir gabarito travão de mão pneumático para B (questoes 411 e 434)
</commit_message>
<xml_diff>
--- a/questoes sem rep.xlsx
+++ b/questoes sem rep.xlsx
@@ -18813,7 +18813,7 @@
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>b</t>
         </is>
       </c>
       <c r="H333" t="inlineStr">
@@ -18823,12 +18823,12 @@
       </c>
       <c r="I333" t="inlineStr">
         <is>
-          <t>gabarito_testescam</t>
+          <t>corrigida</t>
         </is>
       </c>
       <c r="J333" t="inlineStr">
         <is>
-          <t>Importado IMT rel_2 | Gabarito IMT pendente | Gabarito TestesCAM (exato 100%, opcao_texto)</t>
+          <t>Gabarito corrigido manualmente: B (ação pneumática)</t>
         </is>
       </c>
       <c r="K333" t="inlineStr">
@@ -20133,7 +20133,7 @@
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>b</t>
         </is>
       </c>
       <c r="H355" t="inlineStr">
@@ -20143,12 +20143,12 @@
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t>gabarito_testescam</t>
+          <t>corrigida</t>
         </is>
       </c>
       <c r="J355" t="inlineStr">
         <is>
-          <t>Importado IMT rel_2 | Gabarito IMT pendente | Gabarito TestesCAM (fuzzy 75%, opcao_texto)</t>
+          <t>Gabarito corrigido manualmente: B (ação pneumática)</t>
         </is>
       </c>
       <c r="K355" t="inlineStr">

</xml_diff>